<commit_message>
Adicionados novos fornecedores de atributos SCAP.
</commit_message>
<xml_diff>
--- a/Atributos no Autenticação.Gov/Atributos.xlsx
+++ b/Atributos no Autenticação.Gov/Atributos.xlsx
@@ -8,10 +8,10 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Atributos" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="CMD para cidadãos estrangeiros " sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="Fornecedores SCAP" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="F.A.Q." sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Atributos" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="CMD para cidadãos estrangeiros " sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Fornecedores SCAP" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="F.A.Q." sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,18 +25,16 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author> </author>
+    <author>Unknown Author</author>
   </authors>
   <commentList>
     <comment ref="A14" authorId="0">
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Considerar a utilização do atributo http://interop.gov.pt/MDC/Cidadao/DataValidadeDoc se o objectivo é obter a validade do documento e não a validade da CMD, ler observações e comentários.</t>
         </r>
@@ -46,11 +44,9 @@
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Considerar a utilização do atributo http://interop.gov.pt/MDC/Cidadao/DataValidadeDoc se o objectivo é obter a validade do documento e não a validade da CMD, ler observações e comentários.</t>
         </r>
@@ -60,11 +56,9 @@
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Anteriormente designado por http://interop.gov.pt/SCCC</t>
         </r>
@@ -74,11 +68,9 @@
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Considerar a utilização do atributo http://interop.gov.pt/MDC/Cidadao/DataValidadeDoc se o objectivo é obter a validade do documento e não a validade da CMD, ler observações e comentários.</t>
         </r>
@@ -88,11 +80,9 @@
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Considerar a utilização do atributo http://interop.gov.pt/MDC/Cidadao/DataValidadeDoc se o objectivo é obter a validade do documento e não a validade da CMD, ler observações e comentários.</t>
         </r>
@@ -102,11 +92,9 @@
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
-            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">Considerar a utilização do atributo http://interop.gov.pt/MDC/Cidadao/DataValidadeDoc se o objectivo é obter a validade do documento e não a validade da CMD, ler observações e comentários.</t>
         </r>
@@ -116,8 +104,33 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="D7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">TR:     - Título de residência
+PAS    - Passaporte
+CR:    - Cartão de residência
+DR:    - Certificado de autorização de residência</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1176" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1194" uniqueCount="610">
   <si>
     <t xml:space="preserve">Mecanismo Autenticação</t>
   </si>
@@ -1895,7 +1908,18 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> </t>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DR:</t>
     </r>
   </si>
   <si>
@@ -2069,6 +2093,51 @@
   </si>
   <si>
     <t xml:space="preserve">OMV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banco de Portugal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BdP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Instituto da Segurança Social, I.P.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem dos Arquitectos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OARQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem dos Engenheiros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OENG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordem dos Fisioterapeutas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OFisioterapeutas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONotarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCAP Autárquico - Administração Eleitorial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universidade da Beira Interior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UBI</t>
   </si>
   <si>
     <t xml:space="preserve">NOTA: Para obter os atributos disponíveis por mecanismo de autenticação, deverá ser utilizada a funcionalidade de filtragem na folha excel.</t>
@@ -2483,7 +2552,7 @@
     <t xml:space="preserve">Cidadão português </t>
   </si>
   <si>
-    <t xml:space="preserve">Cidadão estrangeiro (título de residência, passaporte, cartão de residência)</t>
+    <t xml:space="preserve">Cidadão estrangeiro (título de residência, passaporte, cartão de residência, certificado de autorização de residência)</t>
   </si>
   <si>
     <t xml:space="preserve">​http://interop.gov.pt/MDC/Cidadao/DocType</t>
@@ -2599,7 +2668,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2637,6 +2706,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -2761,7 +2835,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2838,11 +2912,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2874,6 +2948,14 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2882,11 +2964,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2902,11 +2984,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="15" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2922,7 +3004,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="15" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2940,6 +3022,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFD9D9D9"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2947,21 +3030,22 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF3C3C3C"/>
-          <bgColor rgb="FFFCFCFC"/>
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3049,8 +3133,114 @@
 </table>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -3066,7 +3256,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="81.57"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="18.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="4" customFormat="true" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -3293,7 +3483,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
         <v>7</v>
       </c>
@@ -3316,7 +3506,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>7</v>
       </c>
@@ -3336,7 +3526,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>53</v>
       </c>
@@ -3356,7 +3546,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="112.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>7</v>
       </c>
@@ -3376,7 +3566,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>60</v>
       </c>
@@ -3453,7 +3643,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>53</v>
       </c>
@@ -3473,7 +3663,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="31.3" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>65</v>
       </c>
@@ -3533,7 +3723,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="30" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="31.3" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>65</v>
       </c>
@@ -3653,7 +3843,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
         <v>60</v>
       </c>
@@ -3673,7 +3863,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
         <v>60</v>
       </c>
@@ -3693,7 +3883,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
         <v>60</v>
       </c>
@@ -3753,7 +3943,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="16.4" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>118</v>
       </c>
@@ -5463,7 +5653,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
         <v>349</v>
       </c>
@@ -5483,7 +5673,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="1" t="s">
         <v>349</v>
       </c>
@@ -5503,7 +5693,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="1" t="s">
         <v>349</v>
       </c>
@@ -5523,7 +5713,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="1" t="s">
         <v>349</v>
       </c>
@@ -5543,7 +5733,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="1" t="s">
         <v>349</v>
       </c>
@@ -5563,7 +5753,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="1" t="s">
         <v>349</v>
       </c>
@@ -5583,7 +5773,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="s">
         <v>7</v>
       </c>
@@ -5604,7 +5794,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="1" t="s">
         <v>7</v>
       </c>
@@ -5624,7 +5814,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="1" t="s">
         <v>7</v>
       </c>
@@ -5647,7 +5837,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="1" t="s">
         <v>7</v>
       </c>
@@ -5668,7 +5858,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="1" t="s">
         <v>7</v>
       </c>
@@ -5689,7 +5879,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="1" t="s">
         <v>7</v>
       </c>
@@ -5710,7 +5900,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="1" t="s">
         <v>7</v>
       </c>
@@ -5730,7 +5920,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="1" t="s">
         <v>7</v>
       </c>
@@ -5774,7 +5964,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="1" t="s">
         <v>7</v>
       </c>
@@ -5795,7 +5985,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="1" t="s">
         <v>7</v>
       </c>
@@ -5816,7 +6006,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="1" t="s">
         <v>7</v>
       </c>
@@ -5837,7 +6027,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="1" t="s">
         <v>7</v>
       </c>
@@ -5858,7 +6048,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="1" t="s">
         <v>7</v>
       </c>
@@ -5879,7 +6069,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="s">
         <v>7</v>
       </c>
@@ -5900,7 +6090,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="1" t="s">
         <v>7</v>
       </c>
@@ -5921,7 +6111,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="1" t="s">
         <v>7</v>
       </c>
@@ -5942,7 +6132,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="1" t="s">
         <v>7</v>
       </c>
@@ -5965,7 +6155,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="147" s="6" customFormat="true" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" s="6" customFormat="true" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="5" t="s">
         <v>7</v>
       </c>
@@ -6348,7 +6538,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="1" t="s">
         <v>60</v>
       </c>
@@ -6551,7 +6741,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="240" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="225.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="1" t="s">
         <v>7</v>
       </c>
@@ -6574,7 +6764,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="162.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="1" t="s">
         <v>7</v>
       </c>
@@ -6597,7 +6787,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="1" t="s">
         <v>7</v>
       </c>
@@ -6635,12 +6825,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D57"/>
-  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.17578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="44.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="61.3"/>
@@ -6648,7 +6838,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="74.28"/>
   </cols>
   <sheetData>
-    <row r="1" s="19" customFormat="true" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="19" customFormat="true" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
         <v>517</v>
       </c>
@@ -6662,7 +6852,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
         <v>520</v>
       </c>
@@ -6673,7 +6863,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
         <v>522</v>
       </c>
@@ -6684,7 +6874,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
         <v>17</v>
       </c>
@@ -6695,7 +6885,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
         <v>524</v>
       </c>
@@ -6706,7 +6896,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
         <v>525</v>
       </c>
@@ -6717,7 +6907,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>112</v>
       </c>
@@ -6731,7 +6921,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>115</v>
       </c>
@@ -6745,7 +6935,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>117</v>
       </c>
@@ -6759,7 +6949,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="s">
         <v>530</v>
       </c>
@@ -6773,7 +6963,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
         <v>533</v>
       </c>
@@ -6787,7 +6977,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
         <v>487</v>
       </c>
@@ -6798,7 +6988,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
         <v>535</v>
       </c>
@@ -6809,7 +6999,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
         <v>536</v>
       </c>
@@ -6820,7 +7010,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
         <v>58</v>
       </c>
@@ -6834,7 +7024,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
         <v>538</v>
       </c>
@@ -6848,7 +7038,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
         <v>540</v>
       </c>
@@ -7070,16 +7260,17 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B22"/>
+  <sheetFormatPr defaultColWidth="9.17578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="94.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="31.83"/>
@@ -7187,6 +7378,78 @@
       </c>
       <c r="B13" s="29" t="s">
         <v>567</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30" t="s">
+        <v>568</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="30" t="s">
+        <v>570</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="30" t="s">
+        <v>129</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="30" t="s">
+        <v>573</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="30" t="s">
+        <v>575</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="30" t="s">
+        <v>577</v>
+      </c>
+      <c r="B19" s="31" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="30" t="s">
+        <v>580</v>
+      </c>
+      <c r="B21" s="31" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="16.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="30" t="s">
+        <v>581</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>582</v>
       </c>
     </row>
   </sheetData>
@@ -7201,208 +7464,208 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A42"/>
-  <sheetFormatPr defaultColWidth="8.6015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.62109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="253.42"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="30" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="31"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="32" t="s">
-        <v>569</v>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="32" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="33"/>
+    </row>
+    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="34" t="s">
+        <v>584</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="33"/>
+      <c r="A4" s="35"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="34" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="34" t="s">
-        <v>572</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34" t="s">
-        <v>576</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34" t="s">
-        <v>577</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34" t="s">
-        <v>578</v>
+        <v>585</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="36" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="36" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="36" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="36" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="36" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="36" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="36" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="36" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
+      <c r="A14" s="36"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="35" t="s">
-        <v>579</v>
+      <c r="A15" s="37" t="s">
+        <v>594</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36"/>
+      <c r="A16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37" t="s">
-        <v>581</v>
+        <v>595</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="39" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="40" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37" t="s">
-        <v>582</v>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="39" t="s">
+        <v>597</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38" t="s">
-        <v>583</v>
+      <c r="A21" s="40" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38" t="s">
+      <c r="A22" s="40" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38" t="s">
+      <c r="A23" s="40" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="37" t="s">
-        <v>584</v>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38" t="s">
+      <c r="A25" s="40" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="37" t="s">
-        <v>585</v>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39" t="s">
+        <v>600</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="38" t="s">
+      <c r="A27" s="40" t="s">
         <v>475</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="38" t="s">
+      <c r="A28" s="40" t="s">
         <v>479</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="38" t="s">
+      <c r="A29" s="40" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="38" t="s">
+      <c r="A30" s="40" t="s">
         <v>485</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="38"/>
+      <c r="A31" s="40"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="39" t="s">
-        <v>586</v>
+      <c r="A32" s="41" t="s">
+        <v>601</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="38" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="38" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="40" t="s">
-        <v>589</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="40" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="40" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="42" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>590</v>
+        <v>605</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="38" t="s">
-        <v>591</v>
+      <c r="A38" s="40" t="s">
+        <v>606</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="38" t="s">
-        <v>592</v>
+      <c r="A39" s="40" t="s">
+        <v>607</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="38" t="s">
-        <v>593</v>
+      <c r="A40" s="40" t="s">
+        <v>608</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="38" t="s">
-        <v>594</v>
+      <c r="A41" s="40" t="s">
+        <v>609</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="38"/>
+      <c r="A42" s="40"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>